<commit_message>
Refined Schedule Viewer: 40% default zoom, backdrop exit, and Student Portal fullscreen support.
</commit_message>
<xml_diff>
--- a/static/assets/room_template.xlsx
+++ b/static/assets/room_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WFH\jeremy\CvSU_Scheduling_System\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Documents\CvSU_Scheduling_System-Version-2 - antigravity_2_claude - Copy\static\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C0D6737-6D35-4095-BB9F-712DE5D380C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4629A760-B1C4-45CE-A5FB-79C56CB099DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1200" windowWidth="12990" windowHeight="15000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Infotech" sheetId="1" r:id="rId1"/>
@@ -25,6 +25,9 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="I47NI8+NO9hkF5aAa3fGrEcHYSKRSjDof4JM8+jTiVE="/>
@@ -61,6 +64,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Century Gothic"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> (046) 437-9505 / </t>
     </r>
@@ -69,6 +73,8 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Wingdings 2"/>
+        <family val="1"/>
+        <charset val="2"/>
       </rPr>
       <t>7</t>
     </r>
@@ -77,6 +83,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Century Gothic"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> (046) 437-6659</t>
     </r>
@@ -224,7 +231,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -257,6 +264,7 @@
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -268,15 +276,18 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Narrow"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -284,6 +295,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Narrow"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -291,12 +303,14 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Narrow"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Narrow"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -304,6 +318,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Narrow"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -311,6 +326,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Narrow"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -318,17 +334,34 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Narrow"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Black"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Wingdings 2"/>
+      <family val="1"/>
+      <charset val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Century Gothic"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -504,24 +537,24 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -540,14 +573,14 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -594,158 +627,6 @@
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1123950" cy="1123950"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="image1.jpg">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BA2C685A-BAA5-4F1F-A733-C31D5A42C09E}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="1123950" cy="1123950"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>638175</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1123950" cy="1123950"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="image1.jpg">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E4EB2D23-6959-466B-88DE-F39FFE7A7A29}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4276725" y="1123950"/>
-          <a:ext cx="1123950" cy="1123950"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1009650</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1123950" cy="1123950"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="image1.jpg">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{71640D13-CDEF-4C08-B68C-61A371AF0168}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3543300" y="2619375"/>
-          <a:ext cx="1123950" cy="1123950"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>209550</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1123950" cy="1123950"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="image1.jpg">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C42EB2B-A480-426B-B152-413BF3EF3867}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4953000" y="2124075"/>
-          <a:ext cx="1123950" cy="1123950"/>
-        </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
@@ -997,7 +878,7 @@
     </row>
     <row r="2" spans="1:26" ht="12" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="27" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="28"/>
@@ -1027,7 +908,7 @@
     </row>
     <row r="3" spans="1:26" ht="15" customHeight="1">
       <c r="A3" s="1"/>
-      <c r="B3" s="42" t="s">
+      <c r="B3" s="29" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="28"/>
@@ -1057,7 +938,7 @@
     </row>
     <row r="4" spans="1:26" ht="12" customHeight="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="27" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="28"/>
@@ -1087,7 +968,7 @@
     </row>
     <row r="5" spans="1:26" ht="12" customHeight="1">
       <c r="A5" s="1"/>
-      <c r="B5" s="41" t="s">
+      <c r="B5" s="27" t="s">
         <v>3</v>
       </c>
       <c r="C5" s="28"/>
@@ -1117,7 +998,7 @@
     </row>
     <row r="6" spans="1:26" ht="12" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="43" t="s">
+      <c r="B6" s="30" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="28"/>
@@ -1147,7 +1028,7 @@
     </row>
     <row r="7" spans="1:26" ht="12" customHeight="1">
       <c r="A7" s="1"/>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="31" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="28"/>
@@ -1177,7 +1058,7 @@
     </row>
     <row r="8" spans="1:26" ht="12" customHeight="1">
       <c r="A8" s="1"/>
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="31" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="28"/>
@@ -2325,16 +2206,16 @@
     </row>
     <row r="46" spans="1:26" ht="17.25" customHeight="1">
       <c r="A46" s="1"/>
-      <c r="B46" s="27" t="s">
+      <c r="B46" s="41" t="s">
         <v>46</v>
       </c>
       <c r="C46" s="28"/>
       <c r="D46" s="20"/>
-      <c r="E46" s="29" t="s">
+      <c r="E46" s="42" t="s">
         <v>47</v>
       </c>
       <c r="F46" s="28"/>
-      <c r="G46" s="30" t="s">
+      <c r="G46" s="43" t="s">
         <v>48</v>
       </c>
       <c r="H46" s="28"/>
@@ -2362,11 +2243,11 @@
       <c r="B47" s="28"/>
       <c r="C47" s="28"/>
       <c r="D47" s="22"/>
-      <c r="E47" s="31" t="s">
+      <c r="E47" s="32" t="s">
         <v>49</v>
       </c>
       <c r="F47" s="28"/>
-      <c r="G47" s="32" t="s">
+      <c r="G47" s="33" t="s">
         <v>50</v>
       </c>
       <c r="H47" s="28"/>
@@ -2508,10 +2389,7 @@
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
-      <c r="G52" s="34">
-        <f>B10</f>
-        <v>0</v>
-      </c>
+      <c r="G52" s="34"/>
       <c r="H52" s="28"/>
       <c r="I52" s="1"/>
       <c r="J52" s="1"/>
@@ -2646,12 +2524,12 @@
     </row>
     <row r="57" spans="1:26" ht="12.75" customHeight="1">
       <c r="A57" s="1"/>
-      <c r="B57" s="27"/>
+      <c r="B57" s="41"/>
       <c r="C57" s="28"/>
       <c r="D57" s="20"/>
-      <c r="E57" s="29"/>
+      <c r="E57" s="42"/>
       <c r="F57" s="28"/>
-      <c r="G57" s="30"/>
+      <c r="G57" s="43"/>
       <c r="H57" s="28"/>
       <c r="I57" s="1"/>
       <c r="J57" s="1"/>
@@ -2677,9 +2555,9 @@
       <c r="B58" s="28"/>
       <c r="C58" s="28"/>
       <c r="D58" s="22"/>
-      <c r="E58" s="31"/>
+      <c r="E58" s="32"/>
       <c r="F58" s="28"/>
-      <c r="G58" s="32"/>
+      <c r="G58" s="33"/>
       <c r="H58" s="28"/>
       <c r="I58" s="1"/>
       <c r="J58" s="1"/>
@@ -29078,11 +28956,11 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B57:C58"/>
+    <mergeCell ref="E57:F57"/>
+    <mergeCell ref="G57:H57"/>
+    <mergeCell ref="E58:F58"/>
+    <mergeCell ref="G58:H58"/>
     <mergeCell ref="B7:H7"/>
     <mergeCell ref="B8:H8"/>
     <mergeCell ref="E47:F47"/>
@@ -29095,19 +28973,20 @@
     <mergeCell ref="B46:C47"/>
     <mergeCell ref="E46:F46"/>
     <mergeCell ref="G46:H46"/>
-    <mergeCell ref="B57:C58"/>
-    <mergeCell ref="E57:F57"/>
-    <mergeCell ref="G57:H57"/>
-    <mergeCell ref="E58:F58"/>
-    <mergeCell ref="G58:H58"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B6:H6"/>
   </mergeCells>
+  <phoneticPr fontId="19" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="B7" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="B8" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.11811023622047245" right="0.11811023622047245" top="0.74803149606299213" bottom="0.51181102362204722" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="85" pageOrder="overThenDown" orientation="portrait"/>
-  <drawing r:id="rId3"/>
+  <pageSetup paperSize="9" scale="85" pageOrder="overThenDown" orientation="portrait" r:id="rId3"/>
+  <drawing r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>